<commit_message>
Sync planning SharePoint : S38
</commit_message>
<xml_diff>
--- a/Plannings 2026 S38.xlsx
+++ b/Plannings 2026 S38.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30431"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
@@ -17,8 +17,11 @@
     <sheet name="Résultats par salarié" sheetId="2" r:id="rId2"/>
     <sheet name="Informations" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -37,315 +40,339 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="119">
   <si>
+    <t>Septembre-2026</t>
+  </si>
+  <si>
+    <t>Sem 38</t>
+  </si>
+  <si>
+    <t>C. PADEL // EDF</t>
+  </si>
+  <si>
+    <t>INVENTAIRE // C. PADEL // EDF</t>
+  </si>
+  <si>
+    <t>C, PADEL</t>
+  </si>
+  <si>
+    <t>C. PADEL // EDF // P25M</t>
+  </si>
+  <si>
+    <t>EDF // ANNIV</t>
+  </si>
+  <si>
+    <t>ANNIV</t>
+  </si>
+  <si>
+    <t>Nom / Prénom</t>
+  </si>
+  <si>
+    <t>14 Lu</t>
+  </si>
+  <si>
+    <t>15 Ma</t>
+  </si>
+  <si>
+    <t>16 Me</t>
+  </si>
+  <si>
+    <t>17 Je</t>
+  </si>
+  <si>
+    <t>18 Ve</t>
+  </si>
+  <si>
+    <t>19 Sa</t>
+  </si>
+  <si>
+    <t>20 Di</t>
+  </si>
+  <si>
+    <t>BARON Corentin</t>
+  </si>
+  <si>
+    <t>BONNET Mateo</t>
+  </si>
+  <si>
+    <t>EDF-C</t>
+  </si>
+  <si>
+    <t>13:45/17:30</t>
+  </si>
+  <si>
+    <t>09:00/13:00</t>
+  </si>
+  <si>
+    <t>BOULARDET Lucas</t>
+  </si>
+  <si>
+    <t>CARRERE Peïo</t>
+  </si>
+  <si>
+    <t>INVEN</t>
+  </si>
+  <si>
+    <t>VDC</t>
+  </si>
+  <si>
+    <t>EIA</t>
+  </si>
+  <si>
+    <t>08:15/09:45</t>
+  </si>
+  <si>
+    <t>09:45/18:00</t>
+  </si>
+  <si>
+    <t>16:00/24:00</t>
+  </si>
+  <si>
+    <t>15:45/17:45</t>
+  </si>
+  <si>
+    <t>08:45/17:30</t>
+  </si>
+  <si>
+    <t>09:45/15:00</t>
+  </si>
+  <si>
+    <t>17:45/24:00</t>
+  </si>
+  <si>
+    <t>CASTELLON Pascaline</t>
+  </si>
+  <si>
+    <t>CONRAD - stage David</t>
+  </si>
+  <si>
+    <t>11:45/18:30</t>
+  </si>
+  <si>
+    <t>16:15/19:30</t>
+  </si>
+  <si>
+    <t>11:45/21:30</t>
+  </si>
+  <si>
+    <t>11:45/22:00</t>
+  </si>
+  <si>
+    <t>09:30/15:30</t>
+  </si>
+  <si>
+    <t>CRUZEL Quentin</t>
+  </si>
+  <si>
+    <t>18:00/24:00</t>
+  </si>
+  <si>
+    <t>16:00/23:30</t>
+  </si>
+  <si>
+    <t>DE NOUEL Maxime</t>
+  </si>
+  <si>
+    <t>C-PAD</t>
+  </si>
+  <si>
+    <t>15:30/17:30</t>
+  </si>
+  <si>
+    <t>11:45/13:45</t>
+  </si>
+  <si>
+    <t>09:45/11:45</t>
+  </si>
+  <si>
+    <t>09:15/10:15</t>
+  </si>
+  <si>
+    <t>15:30/22:30</t>
+  </si>
+  <si>
+    <t>17:30/22:30</t>
+  </si>
+  <si>
+    <t>14:30/17:30</t>
+  </si>
+  <si>
+    <t>10:15/12:15</t>
+  </si>
+  <si>
+    <t>13:45/17:45</t>
+  </si>
+  <si>
+    <t>13:45/15:45</t>
+  </si>
+  <si>
+    <t>DIVIEN Yohan</t>
+  </si>
+  <si>
+    <t>DONAER Nicolas</t>
+  </si>
+  <si>
+    <t>17:15/19:15</t>
+  </si>
+  <si>
+    <t>13:30/14:00</t>
+  </si>
+  <si>
+    <t>11:45/17:15</t>
+  </si>
+  <si>
+    <t>09:00/09:30</t>
+  </si>
+  <si>
+    <t>EDF-B</t>
+  </si>
+  <si>
+    <t>19:15/24:00</t>
+  </si>
+  <si>
+    <t>14:00/15:30</t>
+  </si>
+  <si>
+    <t>09:30/12:30</t>
+  </si>
+  <si>
+    <t>15:30/16:45</t>
+  </si>
+  <si>
+    <t>16:45/18:45</t>
+  </si>
+  <si>
+    <t>19:45/24:00</t>
+  </si>
+  <si>
+    <t>DOVINA Théo</t>
+  </si>
+  <si>
+    <t>20:00/24:00</t>
+  </si>
+  <si>
+    <t>DUTROUILH Pierre</t>
+  </si>
+  <si>
+    <t>CUP-R</t>
+  </si>
+  <si>
+    <t>11:45/15:45</t>
+  </si>
+  <si>
+    <t>19:00/00:30+</t>
+  </si>
+  <si>
+    <t>15:45/17:30</t>
+  </si>
+  <si>
+    <t>GILBERT Pierre</t>
+  </si>
+  <si>
+    <t>HEBERT Jean Baptiste</t>
+  </si>
+  <si>
+    <t>JARGUEL Thomas</t>
+  </si>
+  <si>
+    <t>KABUNDA NDEKE Marvyn</t>
+  </si>
+  <si>
+    <t>LABEFODE Thomas</t>
+  </si>
+  <si>
+    <t>LOUIBA Yacine</t>
+  </si>
+  <si>
+    <t>18:30/24:00</t>
+  </si>
+  <si>
+    <t>MANGIN Etienne</t>
+  </si>
+  <si>
+    <t>MOSTEFA Yanis</t>
+  </si>
+  <si>
+    <t>13:30/19:30</t>
+  </si>
+  <si>
+    <t>09:30/10:15</t>
+  </si>
+  <si>
+    <t>19:30/21:30</t>
+  </si>
+  <si>
+    <t>12:15/12:45</t>
+  </si>
+  <si>
+    <t>PISTORE Remi</t>
+  </si>
+  <si>
+    <t>PUJOL Mathieu</t>
+  </si>
+  <si>
+    <t>EDF-A</t>
+  </si>
+  <si>
+    <t>09:45/17:45</t>
+  </si>
+  <si>
+    <t>11:00/17:45</t>
+  </si>
+  <si>
+    <t>09:45/15:45</t>
+  </si>
+  <si>
+    <t>08:45/09:45</t>
+  </si>
+  <si>
+    <t>09:45/17:30</t>
+  </si>
+  <si>
+    <t>RABII Mehdi</t>
+  </si>
+  <si>
+    <t>13:30/17:30</t>
+  </si>
+  <si>
+    <t>17:30/22:20</t>
+  </si>
+  <si>
+    <t>SANGARNE Enzo</t>
+  </si>
+  <si>
+    <t>TOPPAN Mattis</t>
+  </si>
+  <si>
+    <t>17:30/24:00</t>
+  </si>
+  <si>
+    <t>VASSANT Tiffany</t>
+  </si>
+  <si>
     <t>Planning des salariés du 14/09/2026 au 20/09/2026</t>
   </si>
   <si>
-    <t>Septembre-2026</t>
-  </si>
-  <si>
-    <t>Sem 38</t>
-  </si>
-  <si>
-    <t>Nom / Prénom</t>
-  </si>
-  <si>
-    <t>14 Lu</t>
-  </si>
-  <si>
-    <t>15 Ma</t>
-  </si>
-  <si>
-    <t>16 Me</t>
-  </si>
-  <si>
-    <t>17 Je</t>
-  </si>
-  <si>
-    <t>18 Ve</t>
-  </si>
-  <si>
-    <t>19 Sa</t>
-  </si>
-  <si>
-    <t>20 Di</t>
-  </si>
-  <si>
-    <t>BARON Corentin</t>
-  </si>
-  <si>
-    <t>BONNET Mateo</t>
-  </si>
-  <si>
-    <t>EDF-C</t>
-  </si>
-  <si>
-    <t>13:45/17:30</t>
-  </si>
-  <si>
-    <t>09:00/13:00</t>
-  </si>
-  <si>
-    <t>BOULARDET Lucas</t>
-  </si>
-  <si>
-    <t>CARRERE Peïo</t>
-  </si>
-  <si>
-    <t>INVEN</t>
-  </si>
-  <si>
-    <t>VDC</t>
-  </si>
-  <si>
-    <t>EIA</t>
-  </si>
-  <si>
-    <t>08:15/09:45</t>
-  </si>
-  <si>
-    <t>09:45/18:00</t>
-  </si>
-  <si>
-    <t>16:00/24:00</t>
-  </si>
-  <si>
-    <t>15:45/17:45</t>
-  </si>
-  <si>
-    <t>08:45/17:30</t>
-  </si>
-  <si>
-    <t>09:45/15:00</t>
-  </si>
-  <si>
-    <t>17:45/24:00</t>
-  </si>
-  <si>
-    <t>CASTELLON Pascaline</t>
-  </si>
-  <si>
-    <t>CONRAD - stage David</t>
-  </si>
-  <si>
-    <t>11:45/18:30</t>
-  </si>
-  <si>
-    <t>11:45/21:30</t>
-  </si>
-  <si>
-    <t>11:45/22:00</t>
-  </si>
-  <si>
-    <t>09:30/15:30</t>
-  </si>
-  <si>
-    <t>CRUZEL Quentin</t>
-  </si>
-  <si>
-    <t>18:00/24:00</t>
-  </si>
-  <si>
-    <t>16:00/23:30</t>
-  </si>
-  <si>
-    <t>DE NOUEL Maxime</t>
-  </si>
-  <si>
-    <t>C-PAD</t>
-  </si>
-  <si>
-    <t>15:30/17:30</t>
-  </si>
-  <si>
-    <t>11:45/13:45</t>
-  </si>
-  <si>
-    <t>09:45/11:45</t>
-  </si>
-  <si>
-    <t>09:15/10:15</t>
-  </si>
-  <si>
-    <t>15:30/22:30</t>
-  </si>
-  <si>
-    <t>17:30/22:30</t>
-  </si>
-  <si>
-    <t>14:30/17:30</t>
-  </si>
-  <si>
-    <t>10:15/12:15</t>
-  </si>
-  <si>
-    <t>13:45/17:45</t>
-  </si>
-  <si>
-    <t>13:45/15:45</t>
-  </si>
-  <si>
-    <t>DIVIEN Yohan</t>
-  </si>
-  <si>
-    <t>DONAER Nicolas</t>
-  </si>
-  <si>
-    <t>17:15/19:15</t>
-  </si>
-  <si>
-    <t>13:30/14:00</t>
-  </si>
-  <si>
-    <t>11:45/17:15</t>
-  </si>
-  <si>
-    <t>09:00/09:30</t>
-  </si>
-  <si>
-    <t>EDF-B</t>
-  </si>
-  <si>
-    <t>19:15/24:00</t>
-  </si>
-  <si>
-    <t>14:00/15:30</t>
-  </si>
-  <si>
-    <t>09:30/12:30</t>
-  </si>
-  <si>
-    <t>15:30/16:45</t>
-  </si>
-  <si>
-    <t>16:45/18:45</t>
-  </si>
-  <si>
-    <t>19:45/24:00</t>
-  </si>
-  <si>
-    <t>DOVINA Théo</t>
-  </si>
-  <si>
-    <t>20:00/24:00</t>
-  </si>
-  <si>
-    <t>DUTROUILH Pierre</t>
-  </si>
-  <si>
-    <t>CUP-R</t>
-  </si>
-  <si>
-    <t>11:45/15:45</t>
-  </si>
-  <si>
-    <t>19:00/00:30+</t>
+    <t>Jour de référence : 20/09/2026</t>
+  </si>
+  <si>
+    <t>Du 14/09/2026 au 20/09/2026</t>
+  </si>
+  <si>
+    <t>COMMERCIAL DEDIES</t>
+  </si>
+  <si>
+    <t>ARBITRAGE</t>
+  </si>
+  <si>
+    <t>ANNIVERSAIRE</t>
+  </si>
+  <si>
+    <t>FORMATION</t>
   </si>
   <si>
     <t>FREIXEDAS-BERENGUER Maxime</t>
   </si>
   <si>
-    <t>HEBERT Jean Baptiste</t>
-  </si>
-  <si>
-    <t>JARGUEL Thomas</t>
-  </si>
-  <si>
-    <t>KABUNDA NDEKE Marvyn</t>
-  </si>
-  <si>
-    <t>LABEFODE Thomas</t>
-  </si>
-  <si>
-    <t>LOUIBA Yacine</t>
-  </si>
-  <si>
-    <t>18:30/24:00</t>
-  </si>
-  <si>
-    <t>MANGIN Etienne</t>
-  </si>
-  <si>
-    <t>MOSTEFA Yanis</t>
-  </si>
-  <si>
-    <t>ANNIV</t>
-  </si>
-  <si>
-    <t>13:30/19:30</t>
-  </si>
-  <si>
-    <t>09:30/10:15</t>
-  </si>
-  <si>
-    <t>19:30/21:30</t>
-  </si>
-  <si>
-    <t>12:15/12:45</t>
-  </si>
-  <si>
-    <t>PISTORE Remi</t>
-  </si>
-  <si>
-    <t>PUJOL Mathieu</t>
-  </si>
-  <si>
-    <t>EDF-A</t>
-  </si>
-  <si>
-    <t>09:45/17:45</t>
-  </si>
-  <si>
-    <t>11:00/17:45</t>
-  </si>
-  <si>
-    <t>09:45/15:45</t>
-  </si>
-  <si>
-    <t>08:45/09:45</t>
-  </si>
-  <si>
-    <t>09:45/17:30</t>
-  </si>
-  <si>
-    <t>RABII Mehdi</t>
-  </si>
-  <si>
-    <t>13:30/17:30</t>
-  </si>
-  <si>
-    <t>17:30/22:20</t>
-  </si>
-  <si>
-    <t>SANGARNE Enzo</t>
-  </si>
-  <si>
-    <t>TOPPAN Mattis</t>
-  </si>
-  <si>
-    <t>17:30/24:00</t>
-  </si>
-  <si>
-    <t>VASSANT Tiffany</t>
-  </si>
-  <si>
-    <t>Jour de référence : 20/09/2026</t>
-  </si>
-  <si>
-    <t>Du 14/09/2026 au 20/09/2026</t>
-  </si>
-  <si>
-    <t>COMMERCIAL DEDIES</t>
-  </si>
-  <si>
-    <t>ARBITRAGE</t>
-  </si>
-  <si>
-    <t>ANNIVERSAIRE</t>
-  </si>
-  <si>
-    <t>FORMATION</t>
-  </si>
-  <si>
     <t>Société</t>
   </si>
   <si>
@@ -368,30 +395,6 @@
   </si>
   <si>
     <t>04/09/2026 14:58</t>
-  </si>
-  <si>
-    <t>GILBERT Pierre</t>
-  </si>
-  <si>
-    <t>C. PADEL // EDF</t>
-  </si>
-  <si>
-    <t>INVENTAIRE // C. PADEL // EDF</t>
-  </si>
-  <si>
-    <t>C, PADEL</t>
-  </si>
-  <si>
-    <t>C. PADEL // EDF // P25M</t>
-  </si>
-  <si>
-    <t>EDF // ANNIV</t>
-  </si>
-  <si>
-    <t>15:45/17:30</t>
-  </si>
-  <si>
-    <t>16:15/19:30</t>
   </si>
 </sst>
 </file>
@@ -401,7 +404,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[h]:mm"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -438,51 +441,12 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Helvetica"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
-      <name val="Helvetica"/>
-    </font>
-    <font>
-      <b/>
       <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Helvetica"/>
     </font>
     <font>
       <b/>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
-      <name val="Helvetica"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
-      <name val="Helvetica"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
-      <name val="Helvetica"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Helvetica"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
-      <name val="Helvetica"/>
-    </font>
-    <font>
       <sz val="8"/>
       <color rgb="FF000000"/>
       <name val="Helvetica"/>
@@ -774,7 +738,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -785,37 +749,10 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -824,25 +761,10 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -851,28 +773,10 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -917,23 +821,80 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4677,1221 +4638,1229 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H82"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="42.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B1" s="12" t="s">
+    <row r="1" spans="1:8">
+      <c r="B1" s="45" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="B2" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="12" t="s">
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="B3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B3" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="G3" s="15" t="s">
-        <v>116</v>
-      </c>
-      <c r="H3" s="15" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="15" t="s">
+      <c r="C3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="D3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="F3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="H3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="15" t="s">
+    </row>
+    <row r="4" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="B4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="C4" s="6" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="16" t="s">
+      <c r="D4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="19"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="20" t="s">
+      <c r="E4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="21"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="42" t="s">
+      <c r="F4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="42" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" s="22"/>
-    </row>
-    <row r="7" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="23"/>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="43" t="s">
+      <c r="G4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="43" t="s">
+      <c r="H4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="25"/>
-    </row>
-    <row r="8" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="16" t="s">
+    </row>
+    <row r="5" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A5" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="26"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="28"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="20" t="s">
+      <c r="B5" s="37"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
+      <c r="G5" s="38"/>
+      <c r="H5" s="39"/>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="21"/>
-      <c r="C9" s="34" t="s">
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="21" t="s">
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H6" s="9"/>
+    </row>
+    <row r="7" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A7" s="41"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="F9" s="34" t="s">
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="G9" s="21"/>
-      <c r="H9" s="22" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="29"/>
+      <c r="H7" s="11"/>
+    </row>
+    <row r="8" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A8" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="34"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="35"/>
+      <c r="G8" s="35"/>
+      <c r="H8" s="36"/>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="40" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="8"/>
+      <c r="C9" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" s="8"/>
+      <c r="H9" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="43"/>
       <c r="B10" s="1"/>
-      <c r="C10" s="35" t="s">
-        <v>21</v>
+      <c r="C10" s="15" t="s">
+        <v>26</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F10" s="35" t="s">
-        <v>24</v>
+        <v>28</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>29</v>
       </c>
       <c r="G10" s="1"/>
-      <c r="H10" s="30" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="29"/>
+      <c r="H10" s="12" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="43"/>
       <c r="B11" s="1"/>
       <c r="C11" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="G11" s="1"/>
-      <c r="H11" s="30"/>
-    </row>
-    <row r="12" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="23"/>
-      <c r="B12" s="24"/>
-      <c r="C12" s="24" t="s">
-        <v>26</v>
-      </c>
-      <c r="D12" s="24"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="G12" s="24"/>
-      <c r="H12" s="25"/>
-    </row>
-    <row r="13" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" s="26"/>
-      <c r="C13" s="27"/>
-      <c r="D13" s="27"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="27"/>
-      <c r="G13" s="27"/>
-      <c r="H13" s="28"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="20" t="s">
+      <c r="H11" s="12"/>
+    </row>
+    <row r="12" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A12" s="41"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="G12" s="10"/>
+      <c r="H12" s="11"/>
+    </row>
+    <row r="13" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A13" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="34"/>
+      <c r="C13" s="35"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="35"/>
+      <c r="G13" s="35"/>
+      <c r="H13" s="36"/>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="40" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="H14" s="9"/>
+    </row>
+    <row r="15" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A15" s="41"/>
+      <c r="B15" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="H15" s="11"/>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="40" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A17" s="41"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="11" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" s="40" t="s">
+        <v>43</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="8"/>
+      <c r="F18" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="H18" s="9"/>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" s="43"/>
+      <c r="B19" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="E19" s="1"/>
+      <c r="F19" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="H19" s="12"/>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" s="43"/>
+      <c r="B20" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="E20" s="1"/>
+      <c r="F20" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="G20" s="1"/>
+      <c r="H20" s="12"/>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" s="43"/>
+      <c r="B21" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="E21" s="1"/>
+      <c r="F21" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="G21" s="1"/>
+      <c r="H21" s="12"/>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" s="43"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D22" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="E22" s="1"/>
+      <c r="F22" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="G22" s="1"/>
+      <c r="H22" s="12"/>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" s="43"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="D23" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="E23" s="1"/>
+      <c r="F23" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="G23" s="1"/>
+      <c r="H23" s="12"/>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" s="43"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="G24" s="1"/>
+      <c r="H24" s="12"/>
+    </row>
+    <row r="25" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A25" s="41"/>
+      <c r="B25" s="23"/>
+      <c r="C25" s="23"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="C14" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="D14" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="H14" s="22"/>
-    </row>
-    <row r="15" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="23"/>
-      <c r="B15" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" s="24" t="s">
-        <v>118</v>
-      </c>
-      <c r="D15" s="24" t="s">
-        <v>31</v>
-      </c>
-      <c r="E15" s="24" t="s">
-        <v>32</v>
-      </c>
-      <c r="F15" s="24"/>
-      <c r="G15" s="24" t="s">
-        <v>33</v>
-      </c>
-      <c r="H15" s="25"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
-      <c r="H16" s="22" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="23"/>
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="24"/>
-      <c r="H17" s="25" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="B18" s="38" t="s">
-        <v>38</v>
-      </c>
-      <c r="C18" s="42" t="s">
-        <v>38</v>
-      </c>
-      <c r="D18" s="38" t="s">
-        <v>38</v>
-      </c>
-      <c r="E18" s="21"/>
-      <c r="F18" s="38" t="s">
-        <v>38</v>
-      </c>
-      <c r="G18" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="H18" s="22"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="29"/>
-      <c r="B19" s="39" t="s">
-        <v>39</v>
-      </c>
-      <c r="C19" s="41" t="s">
-        <v>40</v>
-      </c>
-      <c r="D19" s="39" t="s">
-        <v>41</v>
-      </c>
-      <c r="E19" s="1"/>
-      <c r="F19" s="39" t="s">
-        <v>42</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H19" s="30"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="29"/>
-      <c r="B20" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="C20" s="44" t="s">
-        <v>38</v>
-      </c>
-      <c r="D20" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="E20" s="1"/>
-      <c r="F20" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="G20" s="1"/>
-      <c r="H20" s="30"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="29"/>
-      <c r="B21" s="41" t="s">
-        <v>44</v>
-      </c>
-      <c r="C21" s="39" t="s">
-        <v>45</v>
-      </c>
-      <c r="D21" s="41" t="s">
-        <v>40</v>
-      </c>
-      <c r="E21" s="1"/>
-      <c r="F21" s="41" t="s">
-        <v>46</v>
-      </c>
-      <c r="G21" s="1"/>
-      <c r="H21" s="30"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="29"/>
-      <c r="B22" s="41"/>
-      <c r="C22" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="D22" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="E22" s="1"/>
-      <c r="F22" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="G22" s="1"/>
-      <c r="H22" s="30"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="29"/>
-      <c r="B23" s="41"/>
-      <c r="C23" s="41" t="s">
-        <v>44</v>
-      </c>
-      <c r="D23" s="41" t="s">
-        <v>47</v>
-      </c>
-      <c r="E23" s="1"/>
-      <c r="F23" s="41" t="s">
-        <v>48</v>
-      </c>
-      <c r="G23" s="1"/>
-      <c r="H23" s="30"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="29"/>
-      <c r="B24" s="41"/>
-      <c r="C24" s="41"/>
-      <c r="D24" s="41"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="36" t="s">
-        <v>20</v>
-      </c>
-      <c r="G24" s="1"/>
-      <c r="H24" s="30"/>
-    </row>
-    <row r="25" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="23"/>
-      <c r="B25" s="43"/>
-      <c r="C25" s="43"/>
-      <c r="D25" s="43"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="37" t="s">
-        <v>24</v>
-      </c>
-      <c r="G25" s="24"/>
-      <c r="H25" s="25"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="B26" s="21"/>
-      <c r="C26" s="21"/>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
-      <c r="F26" s="21"/>
-      <c r="G26" s="42" t="s">
-        <v>13</v>
-      </c>
-      <c r="H26" s="22"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="29"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="11"/>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" s="40" t="s">
+        <v>55</v>
+      </c>
+      <c r="B26" s="8"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H26" s="9"/>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27" s="43"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
-      <c r="G27" s="41" t="s">
-        <v>15</v>
-      </c>
-      <c r="H27" s="30"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="29"/>
+      <c r="G27" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="H27" s="12"/>
+    </row>
+    <row r="28" spans="1:8">
+      <c r="A28" s="43"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
-      <c r="G28" s="40" t="s">
-        <v>13</v>
-      </c>
-      <c r="H28" s="30"/>
-    </row>
-    <row r="29" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="23"/>
-      <c r="B29" s="24"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="24"/>
-      <c r="G29" s="43" t="s">
-        <v>48</v>
-      </c>
-      <c r="H29" s="25"/>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="20" t="s">
-        <v>50</v>
-      </c>
-      <c r="B30" s="42" t="s">
-        <v>13</v>
-      </c>
-      <c r="C30" s="42" t="s">
-        <v>13</v>
-      </c>
-      <c r="D30" s="42" t="s">
-        <v>13</v>
-      </c>
-      <c r="E30" s="21"/>
-      <c r="F30" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="G30" s="42" t="s">
-        <v>13</v>
-      </c>
-      <c r="H30" s="22"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="29"/>
-      <c r="B31" s="41" t="s">
-        <v>51</v>
-      </c>
-      <c r="C31" s="41" t="s">
-        <v>51</v>
-      </c>
-      <c r="D31" s="41" t="s">
-        <v>52</v>
+      <c r="G28" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="H28" s="12"/>
+    </row>
+    <row r="29" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A29" s="41"/>
+      <c r="B29" s="10"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="H29" s="11"/>
+    </row>
+    <row r="30" spans="1:8">
+      <c r="A30" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="B30" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="C30" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="D30" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G30" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H30" s="9"/>
+    </row>
+    <row r="31" spans="1:8">
+      <c r="A31" s="43"/>
+      <c r="B31" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="C31" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="D31" s="21" t="s">
+        <v>58</v>
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G31" s="41" t="s">
-        <v>54</v>
-      </c>
-      <c r="H31" s="30"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="29"/>
+        <v>59</v>
+      </c>
+      <c r="G31" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="H31" s="12"/>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="A32" s="43"/>
       <c r="B32" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D32" s="40" t="s">
-        <v>55</v>
+        <v>24</v>
+      </c>
+      <c r="D32" s="20" t="s">
+        <v>61</v>
       </c>
       <c r="E32" s="1"/>
-      <c r="F32" s="40" t="s">
-        <v>13</v>
-      </c>
-      <c r="G32" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="H32" s="30"/>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="29"/>
+      <c r="F32" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="G32" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="H32" s="12"/>
+    </row>
+    <row r="33" spans="1:8">
+      <c r="A33" s="43"/>
       <c r="B33" s="1" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D33" s="41" t="s">
+        <v>62</v>
+      </c>
+      <c r="D33" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="E33" s="1"/>
+      <c r="F33" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="E33" s="1"/>
-      <c r="F33" s="41" t="s">
-        <v>51</v>
-      </c>
-      <c r="G33" s="41" t="s">
-        <v>58</v>
-      </c>
-      <c r="H33" s="30"/>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="29"/>
+      <c r="G33" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="H33" s="12"/>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34" s="43"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
-      <c r="D34" s="40" t="s">
-        <v>13</v>
+      <c r="D34" s="20" t="s">
+        <v>18</v>
       </c>
       <c r="E34" s="1"/>
-      <c r="F34" s="41"/>
-      <c r="G34" s="41"/>
-      <c r="H34" s="30"/>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="29"/>
+      <c r="F34" s="21"/>
+      <c r="G34" s="21"/>
+      <c r="H34" s="12"/>
+    </row>
+    <row r="35" spans="1:8">
+      <c r="A35" s="43"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
-      <c r="D35" s="41" t="s">
-        <v>59</v>
+      <c r="D35" s="21" t="s">
+        <v>65</v>
       </c>
       <c r="E35" s="1"/>
-      <c r="F35" s="41"/>
-      <c r="G35" s="41"/>
-      <c r="H35" s="30"/>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="29"/>
+      <c r="F35" s="21"/>
+      <c r="G35" s="21"/>
+      <c r="H35" s="12"/>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36" s="43"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
-      <c r="D36" s="40" t="s">
-        <v>55</v>
+      <c r="D36" s="20" t="s">
+        <v>61</v>
       </c>
       <c r="E36" s="1"/>
-      <c r="F36" s="41"/>
-      <c r="G36" s="41"/>
-      <c r="H36" s="30"/>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="29"/>
+      <c r="F36" s="21"/>
+      <c r="G36" s="21"/>
+      <c r="H36" s="12"/>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37" s="43"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
-      <c r="D37" s="41" t="s">
-        <v>60</v>
+      <c r="D37" s="21" t="s">
+        <v>66</v>
       </c>
       <c r="E37" s="1"/>
-      <c r="F37" s="41"/>
-      <c r="G37" s="41"/>
-      <c r="H37" s="30"/>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="29"/>
+      <c r="F37" s="21"/>
+      <c r="G37" s="21"/>
+      <c r="H37" s="12"/>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" s="43"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
       <c r="D38" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="E38" s="1"/>
-      <c r="F38" s="41"/>
-      <c r="G38" s="41"/>
-      <c r="H38" s="30"/>
-    </row>
-    <row r="39" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="31"/>
+      <c r="F38" s="21"/>
+      <c r="G38" s="21"/>
+      <c r="H38" s="12"/>
+    </row>
+    <row r="39" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A39" s="44"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
       <c r="D39" s="1" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="E39" s="1"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="41"/>
-      <c r="H39" s="30"/>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="20" t="s">
-        <v>62</v>
-      </c>
-      <c r="B40" s="21"/>
-      <c r="C40" s="21"/>
-      <c r="D40" s="21"/>
-      <c r="E40" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="F40" s="21"/>
-      <c r="G40" s="21"/>
-      <c r="H40" s="22"/>
-    </row>
-    <row r="41" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="23"/>
-      <c r="B41" s="24"/>
-      <c r="C41" s="24"/>
-      <c r="D41" s="24"/>
-      <c r="E41" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="F41" s="24"/>
-      <c r="G41" s="24"/>
-      <c r="H41" s="25"/>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="B42" s="21"/>
-      <c r="C42" s="21"/>
-      <c r="D42" s="42" t="s">
-        <v>38</v>
-      </c>
-      <c r="E42" s="42" t="s">
-        <v>38</v>
-      </c>
-      <c r="F42" s="45" t="s">
-        <v>65</v>
-      </c>
-      <c r="G42" s="21"/>
-      <c r="H42" s="22"/>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="29"/>
+      <c r="F39" s="21"/>
+      <c r="G39" s="21"/>
+      <c r="H39" s="12"/>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40" s="40" t="s">
+        <v>68</v>
+      </c>
+      <c r="B40" s="8"/>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F40" s="8"/>
+      <c r="G40" s="8"/>
+      <c r="H40" s="9"/>
+    </row>
+    <row r="41" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A41" s="41"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="11"/>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42" s="40" t="s">
+        <v>70</v>
+      </c>
+      <c r="B42" s="8"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="E42" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="F42" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="G42" s="8"/>
+      <c r="H42" s="9"/>
+    </row>
+    <row r="43" spans="1:8">
+      <c r="A43" s="43"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
-      <c r="D43" s="41" t="s">
-        <v>48</v>
-      </c>
-      <c r="E43" s="41" t="s">
-        <v>66</v>
-      </c>
-      <c r="F43" s="46" t="s">
-        <v>67</v>
+      <c r="D43" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="E43" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="F43" s="26" t="s">
+        <v>73</v>
       </c>
       <c r="G43" s="1"/>
-      <c r="H43" s="30"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="29"/>
+      <c r="H43" s="12"/>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="A44" s="43"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
-      <c r="D44" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="E44" s="44" t="s">
-        <v>38</v>
-      </c>
-      <c r="F44" s="46"/>
+      <c r="D44" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="E44" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="F44" s="26"/>
       <c r="G44" s="1"/>
-      <c r="H44" s="30"/>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A45" s="29"/>
+      <c r="H44" s="12"/>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45" s="43"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
-      <c r="D45" s="41" t="s">
-        <v>44</v>
-      </c>
-      <c r="E45" s="39" t="s">
-        <v>117</v>
-      </c>
-      <c r="F45" s="46"/>
+      <c r="D45" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="E45" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="F45" s="26"/>
       <c r="G45" s="1"/>
-      <c r="H45" s="30"/>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A46" s="29"/>
+      <c r="H45" s="12"/>
+    </row>
+    <row r="46" spans="1:8">
+      <c r="A46" s="43"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
-      <c r="D46" s="41"/>
-      <c r="E46" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="F46" s="46"/>
+      <c r="D46" s="21"/>
+      <c r="E46" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="F46" s="26"/>
       <c r="G46" s="1"/>
-      <c r="H46" s="30"/>
-    </row>
-    <row r="47" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="23"/>
-      <c r="B47" s="24"/>
-      <c r="C47" s="24"/>
-      <c r="D47" s="43"/>
-      <c r="E47" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="F47" s="47"/>
-      <c r="G47" s="24"/>
-      <c r="H47" s="25"/>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A48" s="20" t="s">
-        <v>111</v>
-      </c>
-      <c r="B48" s="21"/>
-      <c r="C48" s="21"/>
-      <c r="D48" s="42" t="s">
-        <v>13</v>
-      </c>
-      <c r="E48" s="21"/>
-      <c r="F48" s="21"/>
-      <c r="G48" s="42" t="s">
-        <v>13</v>
-      </c>
-      <c r="H48" s="22"/>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A49" s="29"/>
+      <c r="H46" s="12"/>
+    </row>
+    <row r="47" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A47" s="41"/>
+      <c r="B47" s="10"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="23"/>
+      <c r="E47" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="F47" s="27"/>
+      <c r="G47" s="10"/>
+      <c r="H47" s="11"/>
+    </row>
+    <row r="48" spans="1:8">
+      <c r="A48" s="40" t="s">
+        <v>75</v>
+      </c>
+      <c r="B48" s="8"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="E48" s="8"/>
+      <c r="F48" s="8"/>
+      <c r="G48" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H48" s="9"/>
+    </row>
+    <row r="49" spans="1:8">
+      <c r="A49" s="43"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
-      <c r="D49" s="41" t="s">
-        <v>14</v>
+      <c r="D49" s="21" t="s">
+        <v>19</v>
       </c>
       <c r="E49" s="1"/>
       <c r="F49" s="1"/>
-      <c r="G49" s="41" t="s">
-        <v>15</v>
-      </c>
-      <c r="H49" s="30"/>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A50" s="29"/>
+      <c r="G49" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="H49" s="12"/>
+    </row>
+    <row r="50" spans="1:8">
+      <c r="A50" s="43"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
-      <c r="D50" s="41"/>
+      <c r="D50" s="21"/>
       <c r="E50" s="1"/>
       <c r="F50" s="1"/>
-      <c r="G50" s="40" t="s">
-        <v>13</v>
-      </c>
-      <c r="H50" s="30"/>
-    </row>
-    <row r="51" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="23"/>
-      <c r="B51" s="24"/>
-      <c r="C51" s="24"/>
-      <c r="D51" s="43"/>
-      <c r="E51" s="24"/>
-      <c r="F51" s="24"/>
-      <c r="G51" s="43" t="s">
-        <v>47</v>
-      </c>
-      <c r="H51" s="25"/>
-    </row>
-    <row r="52" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="B52" s="26"/>
-      <c r="C52" s="27"/>
-      <c r="D52" s="27"/>
-      <c r="E52" s="27"/>
-      <c r="F52" s="27"/>
-      <c r="G52" s="27"/>
-      <c r="H52" s="28"/>
-    </row>
-    <row r="53" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="B53" s="26"/>
-      <c r="C53" s="27"/>
-      <c r="D53" s="27"/>
-      <c r="E53" s="27"/>
-      <c r="F53" s="27"/>
-      <c r="G53" s="27"/>
-      <c r="H53" s="28"/>
-    </row>
-    <row r="54" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="B54" s="26"/>
-      <c r="C54" s="27"/>
-      <c r="D54" s="27"/>
-      <c r="E54" s="27"/>
-      <c r="F54" s="27"/>
-      <c r="G54" s="27"/>
-      <c r="H54" s="28"/>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A55" s="20" t="s">
-        <v>72</v>
-      </c>
-      <c r="B55" s="21"/>
-      <c r="C55" s="21"/>
-      <c r="D55" s="21"/>
-      <c r="E55" s="21"/>
-      <c r="F55" s="42" t="s">
-        <v>13</v>
-      </c>
-      <c r="G55" s="21"/>
-      <c r="H55" s="22"/>
-    </row>
-    <row r="56" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="31"/>
+      <c r="G50" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="H50" s="12"/>
+    </row>
+    <row r="51" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A51" s="41"/>
+      <c r="B51" s="10"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="23"/>
+      <c r="E51" s="10"/>
+      <c r="F51" s="10"/>
+      <c r="G51" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="H51" s="11"/>
+    </row>
+    <row r="52" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A52" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B52" s="34"/>
+      <c r="C52" s="35"/>
+      <c r="D52" s="35"/>
+      <c r="E52" s="35"/>
+      <c r="F52" s="35"/>
+      <c r="G52" s="35"/>
+      <c r="H52" s="36"/>
+    </row>
+    <row r="53" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A53" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B53" s="34"/>
+      <c r="C53" s="35"/>
+      <c r="D53" s="35"/>
+      <c r="E53" s="35"/>
+      <c r="F53" s="35"/>
+      <c r="G53" s="35"/>
+      <c r="H53" s="36"/>
+    </row>
+    <row r="54" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A54" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B54" s="34"/>
+      <c r="C54" s="35"/>
+      <c r="D54" s="35"/>
+      <c r="E54" s="35"/>
+      <c r="F54" s="35"/>
+      <c r="G54" s="35"/>
+      <c r="H54" s="36"/>
+    </row>
+    <row r="55" spans="1:8">
+      <c r="A55" s="40" t="s">
+        <v>79</v>
+      </c>
+      <c r="B55" s="8"/>
+      <c r="C55" s="8"/>
+      <c r="D55" s="8"/>
+      <c r="E55" s="8"/>
+      <c r="F55" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="G55" s="8"/>
+      <c r="H55" s="9"/>
+    </row>
+    <row r="56" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A56" s="44"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
       <c r="D56" s="1"/>
       <c r="E56" s="1"/>
-      <c r="F56" s="41" t="s">
-        <v>51</v>
+      <c r="F56" s="21" t="s">
+        <v>57</v>
       </c>
       <c r="G56" s="1"/>
-      <c r="H56" s="30"/>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A57" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="B57" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="C57" s="21"/>
-      <c r="D57" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="E57" s="21"/>
-      <c r="F57" s="21"/>
-      <c r="G57" s="21"/>
-      <c r="H57" s="22"/>
-    </row>
-    <row r="58" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="23"/>
-      <c r="B58" s="24" t="s">
-        <v>74</v>
-      </c>
-      <c r="C58" s="24"/>
-      <c r="D58" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="E58" s="24"/>
-      <c r="F58" s="24"/>
-      <c r="G58" s="24"/>
-      <c r="H58" s="25"/>
-    </row>
-    <row r="59" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="B59" s="26"/>
-      <c r="C59" s="27"/>
-      <c r="D59" s="27"/>
-      <c r="E59" s="27"/>
-      <c r="F59" s="27"/>
-      <c r="G59" s="27"/>
-      <c r="H59" s="28"/>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A60" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="B60" s="21"/>
-      <c r="C60" s="21"/>
-      <c r="D60" s="21"/>
-      <c r="E60" s="21"/>
-      <c r="F60" s="21"/>
-      <c r="G60" s="52" t="s">
-        <v>77</v>
-      </c>
-      <c r="H60" s="22" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A61" s="29"/>
+      <c r="H56" s="12"/>
+    </row>
+    <row r="57" spans="1:8">
+      <c r="A57" s="40" t="s">
+        <v>80</v>
+      </c>
+      <c r="B57" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C57" s="8"/>
+      <c r="D57" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E57" s="8"/>
+      <c r="F57" s="8"/>
+      <c r="G57" s="8"/>
+      <c r="H57" s="9"/>
+    </row>
+    <row r="58" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A58" s="41"/>
+      <c r="B58" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="C58" s="10"/>
+      <c r="D58" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="E58" s="10"/>
+      <c r="F58" s="10"/>
+      <c r="G58" s="10"/>
+      <c r="H58" s="11"/>
+    </row>
+    <row r="59" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A59" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B59" s="34"/>
+      <c r="C59" s="35"/>
+      <c r="D59" s="35"/>
+      <c r="E59" s="35"/>
+      <c r="F59" s="35"/>
+      <c r="G59" s="35"/>
+      <c r="H59" s="36"/>
+    </row>
+    <row r="60" spans="1:8">
+      <c r="A60" s="40" t="s">
+        <v>83</v>
+      </c>
+      <c r="B60" s="8"/>
+      <c r="C60" s="8"/>
+      <c r="D60" s="8"/>
+      <c r="E60" s="8"/>
+      <c r="F60" s="8"/>
+      <c r="G60" s="32" t="s">
+        <v>7</v>
+      </c>
+      <c r="H60" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8">
+      <c r="A61" s="43"/>
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
       <c r="D61" s="1"/>
       <c r="E61" s="1"/>
       <c r="F61" s="1"/>
-      <c r="G61" s="53" t="s">
-        <v>78</v>
-      </c>
-      <c r="H61" s="30" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A62" s="29"/>
+      <c r="G61" s="33" t="s">
+        <v>84</v>
+      </c>
+      <c r="H61" s="12" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8">
+      <c r="A62" s="43"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
       <c r="D62" s="1"/>
       <c r="E62" s="1"/>
       <c r="F62" s="1"/>
       <c r="G62" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H62" s="50" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A63" s="29"/>
+        <v>24</v>
+      </c>
+      <c r="H62" s="30" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8">
+      <c r="A63" s="43"/>
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
       <c r="D63" s="1"/>
       <c r="E63" s="1"/>
       <c r="F63" s="1"/>
       <c r="G63" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="H63" s="49" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A64" s="29"/>
+        <v>86</v>
+      </c>
+      <c r="H63" s="29" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8">
+      <c r="A64" s="43"/>
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
       <c r="D64" s="1"/>
       <c r="E64" s="1"/>
       <c r="F64" s="1"/>
       <c r="G64" s="1"/>
-      <c r="H64" s="32" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A65" s="29"/>
+      <c r="H64" s="13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8">
+      <c r="A65" s="43"/>
       <c r="B65" s="1"/>
       <c r="C65" s="1"/>
       <c r="D65" s="1"/>
       <c r="E65" s="1"/>
       <c r="F65" s="1"/>
       <c r="G65" s="1"/>
-      <c r="H65" s="30" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A66" s="29"/>
+      <c r="H65" s="12" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8">
+      <c r="A66" s="43"/>
       <c r="B66" s="1"/>
       <c r="C66" s="1"/>
       <c r="D66" s="1"/>
       <c r="E66" s="1"/>
       <c r="F66" s="1"/>
       <c r="G66" s="1"/>
-      <c r="H66" s="50" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="67" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="23"/>
-      <c r="B67" s="24"/>
-      <c r="C67" s="24"/>
-      <c r="D67" s="24"/>
-      <c r="E67" s="24"/>
-      <c r="F67" s="24"/>
-      <c r="G67" s="24"/>
-      <c r="H67" s="51" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A68" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="B68" s="21"/>
-      <c r="C68" s="21"/>
-      <c r="D68" s="21"/>
-      <c r="E68" s="21"/>
-      <c r="F68" s="42" t="s">
-        <v>13</v>
-      </c>
-      <c r="G68" s="21"/>
-      <c r="H68" s="22"/>
-    </row>
-    <row r="69" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="23"/>
-      <c r="B69" s="24"/>
-      <c r="C69" s="24"/>
-      <c r="D69" s="24"/>
-      <c r="E69" s="24"/>
-      <c r="F69" s="43" t="s">
-        <v>51</v>
-      </c>
-      <c r="G69" s="24"/>
-      <c r="H69" s="25"/>
-    </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A70" s="20" t="s">
-        <v>83</v>
-      </c>
-      <c r="B70" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="C70" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="D70" s="21"/>
-      <c r="E70" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="F70" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="G70" s="42" t="s">
-        <v>84</v>
-      </c>
-      <c r="H70" s="22"/>
-    </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A71" s="29"/>
+      <c r="H66" s="30" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A67" s="41"/>
+      <c r="B67" s="10"/>
+      <c r="C67" s="10"/>
+      <c r="D67" s="10"/>
+      <c r="E67" s="10"/>
+      <c r="F67" s="10"/>
+      <c r="G67" s="10"/>
+      <c r="H67" s="31" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8">
+      <c r="A68" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="B68" s="8"/>
+      <c r="C68" s="8"/>
+      <c r="D68" s="8"/>
+      <c r="E68" s="8"/>
+      <c r="F68" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="G68" s="8"/>
+      <c r="H68" s="9"/>
+    </row>
+    <row r="69" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A69" s="41"/>
+      <c r="B69" s="10"/>
+      <c r="C69" s="10"/>
+      <c r="D69" s="10"/>
+      <c r="E69" s="10"/>
+      <c r="F69" s="23" t="s">
+        <v>57</v>
+      </c>
+      <c r="G69" s="10"/>
+      <c r="H69" s="11"/>
+    </row>
+    <row r="70" spans="1:8">
+      <c r="A70" s="40" t="s">
+        <v>89</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C70" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D70" s="8"/>
+      <c r="E70" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F70" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G70" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="H70" s="9"/>
+    </row>
+    <row r="71" spans="1:8">
+      <c r="A71" s="43"/>
       <c r="B71" s="1" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="D71" s="1"/>
       <c r="E71" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="G71" s="41" t="s">
-        <v>88</v>
-      </c>
-      <c r="H71" s="30"/>
-    </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A72" s="29"/>
+        <v>93</v>
+      </c>
+      <c r="G71" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="H71" s="12"/>
+    </row>
+    <row r="72" spans="1:8">
+      <c r="A72" s="43"/>
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
       <c r="D72" s="1"/>
       <c r="E72" s="1"/>
-      <c r="F72" s="36" t="s">
-        <v>20</v>
+      <c r="F72" s="16" t="s">
+        <v>25</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H72" s="30"/>
-    </row>
-    <row r="73" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="23"/>
-      <c r="B73" s="24"/>
-      <c r="C73" s="24"/>
-      <c r="D73" s="24"/>
-      <c r="E73" s="24"/>
-      <c r="F73" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="G73" s="24" t="s">
-        <v>89</v>
-      </c>
-      <c r="H73" s="25"/>
-    </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A74" s="20" t="s">
-        <v>90</v>
-      </c>
-      <c r="B74" s="21"/>
-      <c r="C74" s="21"/>
-      <c r="D74" s="21"/>
-      <c r="E74" s="21"/>
-      <c r="F74" s="21"/>
-      <c r="G74" s="21"/>
-      <c r="H74" s="48" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A75" s="29"/>
+      <c r="H72" s="12"/>
+    </row>
+    <row r="73" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A73" s="41"/>
+      <c r="B73" s="10"/>
+      <c r="C73" s="10"/>
+      <c r="D73" s="10"/>
+      <c r="E73" s="10"/>
+      <c r="F73" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="G73" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="H73" s="11"/>
+    </row>
+    <row r="74" spans="1:8">
+      <c r="A74" s="40" t="s">
+        <v>96</v>
+      </c>
+      <c r="B74" s="8"/>
+      <c r="C74" s="8"/>
+      <c r="D74" s="8"/>
+      <c r="E74" s="8"/>
+      <c r="F74" s="8"/>
+      <c r="G74" s="8"/>
+      <c r="H74" s="28" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8">
+      <c r="A75" s="43"/>
       <c r="B75" s="1"/>
       <c r="C75" s="1"/>
       <c r="D75" s="1"/>
       <c r="E75" s="1"/>
       <c r="F75" s="1"/>
       <c r="G75" s="1"/>
-      <c r="H75" s="49" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A76" s="29"/>
+      <c r="H75" s="29" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8">
+      <c r="A76" s="43"/>
       <c r="B76" s="1"/>
       <c r="C76" s="1"/>
       <c r="D76" s="1"/>
       <c r="E76" s="1"/>
       <c r="F76" s="1"/>
       <c r="G76" s="1"/>
-      <c r="H76" s="32" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="77" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="31"/>
+      <c r="H76" s="13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A77" s="44"/>
       <c r="B77" s="1"/>
       <c r="C77" s="1"/>
       <c r="D77" s="1"/>
       <c r="E77" s="1"/>
       <c r="F77" s="1"/>
       <c r="G77" s="1"/>
-      <c r="H77" s="30" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="78" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="16" t="s">
-        <v>93</v>
-      </c>
-      <c r="B78" s="26"/>
-      <c r="C78" s="27"/>
-      <c r="D78" s="27"/>
-      <c r="E78" s="27"/>
-      <c r="F78" s="27"/>
-      <c r="G78" s="27"/>
-      <c r="H78" s="28"/>
-    </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A79" s="20" t="s">
-        <v>94</v>
-      </c>
-      <c r="B79" s="21"/>
-      <c r="C79" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="D79" s="21"/>
-      <c r="E79" s="21"/>
-      <c r="F79" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="G79" s="21"/>
-      <c r="H79" s="22"/>
-    </row>
-    <row r="80" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="23"/>
-      <c r="B80" s="24"/>
-      <c r="C80" s="24" t="s">
-        <v>95</v>
-      </c>
-      <c r="D80" s="24"/>
-      <c r="E80" s="24"/>
-      <c r="F80" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="G80" s="24"/>
-      <c r="H80" s="25"/>
-    </row>
-    <row r="81" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="16" t="s">
-        <v>96</v>
-      </c>
-      <c r="B81" s="26"/>
-      <c r="C81" s="27"/>
-      <c r="D81" s="27"/>
-      <c r="E81" s="27"/>
-      <c r="F81" s="27"/>
-      <c r="G81" s="27"/>
-      <c r="H81" s="28"/>
-    </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B82" s="33"/>
-      <c r="C82" s="33"/>
-      <c r="D82" s="33"/>
-      <c r="E82" s="33"/>
-      <c r="F82" s="33"/>
-      <c r="G82" s="33"/>
-      <c r="H82" s="33"/>
+      <c r="H77" s="12" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A78" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B78" s="34"/>
+      <c r="C78" s="35"/>
+      <c r="D78" s="35"/>
+      <c r="E78" s="35"/>
+      <c r="F78" s="35"/>
+      <c r="G78" s="35"/>
+      <c r="H78" s="36"/>
+    </row>
+    <row r="79" spans="1:8">
+      <c r="A79" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="B79" s="8"/>
+      <c r="C79" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D79" s="8"/>
+      <c r="E79" s="8"/>
+      <c r="F79" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G79" s="8"/>
+      <c r="H79" s="9"/>
+    </row>
+    <row r="80" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A80" s="41"/>
+      <c r="B80" s="10"/>
+      <c r="C80" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="D80" s="10"/>
+      <c r="E80" s="10"/>
+      <c r="F80" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="G80" s="10"/>
+      <c r="H80" s="11"/>
+    </row>
+    <row r="81" spans="1:8" ht="15.75" thickBot="1">
+      <c r="A81" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B81" s="34"/>
+      <c r="C81" s="35"/>
+      <c r="D81" s="35"/>
+      <c r="E81" s="35"/>
+      <c r="F81" s="35"/>
+      <c r="G81" s="35"/>
+      <c r="H81" s="36"/>
+    </row>
+    <row r="82" spans="1:8">
+      <c r="B82" s="42"/>
+      <c r="C82" s="42"/>
+      <c r="D82" s="42"/>
+      <c r="E82" s="42"/>
+      <c r="F82" s="42"/>
+      <c r="G82" s="42"/>
+      <c r="H82" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="B52:H52"/>
-    <mergeCell ref="B53:H53"/>
-    <mergeCell ref="B54:H54"/>
-    <mergeCell ref="B13:H13"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B8:H8"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A9:A12"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="A18:A25"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="A55:A56"/>
+    <mergeCell ref="A57:A58"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A30:A39"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="A42:A47"/>
+    <mergeCell ref="A48:A51"/>
     <mergeCell ref="A79:A80"/>
     <mergeCell ref="B82:H82"/>
     <mergeCell ref="B59:H59"/>
@@ -5901,20 +5870,12 @@
     <mergeCell ref="A68:A69"/>
     <mergeCell ref="A70:A73"/>
     <mergeCell ref="A74:A77"/>
-    <mergeCell ref="A55:A56"/>
-    <mergeCell ref="A57:A58"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="A30:A39"/>
-    <mergeCell ref="A40:A41"/>
-    <mergeCell ref="A42:A47"/>
-    <mergeCell ref="A48:A51"/>
-    <mergeCell ref="A9:A12"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="A18:A25"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B52:H52"/>
+    <mergeCell ref="B53:H53"/>
+    <mergeCell ref="B54:H54"/>
+    <mergeCell ref="B13:H13"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B8:H8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="38" fitToHeight="0" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -5925,499 +5886,499 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="15.75">
       <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B4" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B5" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="6" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="B4" s="46" t="s">
+        <v>104</v>
+      </c>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="B5" s="47" t="s">
+        <v>105</v>
+      </c>
+      <c r="C5" s="47"/>
+      <c r="D5" s="47"/>
+      <c r="E5" s="47"/>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="48" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="49">
+        <v>0</v>
+      </c>
+      <c r="C7" s="49">
+        <v>0</v>
+      </c>
+      <c r="D7" s="49">
+        <v>0</v>
+      </c>
+      <c r="E7" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="48" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="49">
+        <v>0</v>
+      </c>
+      <c r="C8" s="49">
+        <v>0</v>
+      </c>
+      <c r="D8" s="49">
+        <v>0</v>
+      </c>
+      <c r="E8" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="48" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="49">
+        <v>0</v>
+      </c>
+      <c r="C9" s="49">
+        <v>0</v>
+      </c>
+      <c r="D9" s="49">
+        <v>0</v>
+      </c>
+      <c r="E9" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="49">
+        <v>0</v>
+      </c>
+      <c r="C10" s="49">
+        <v>0</v>
+      </c>
+      <c r="D10" s="49">
+        <v>0</v>
+      </c>
+      <c r="E10" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="48" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="49">
+        <v>0</v>
+      </c>
+      <c r="C11" s="49">
+        <v>0</v>
+      </c>
+      <c r="D11" s="49">
+        <v>0</v>
+      </c>
+      <c r="E11" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="48" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="49">
+        <v>0</v>
+      </c>
+      <c r="C12" s="49">
+        <v>0</v>
+      </c>
+      <c r="D12" s="49">
+        <v>0</v>
+      </c>
+      <c r="E12" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="48" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="49">
+        <v>0</v>
+      </c>
+      <c r="C13" s="49">
+        <v>0</v>
+      </c>
+      <c r="D13" s="49">
+        <v>0</v>
+      </c>
+      <c r="E13" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="B14" s="49">
+        <v>0</v>
+      </c>
+      <c r="C14" s="49">
+        <v>0</v>
+      </c>
+      <c r="D14" s="49">
+        <v>0</v>
+      </c>
+      <c r="E14" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="48" t="s">
+        <v>55</v>
+      </c>
+      <c r="B15" s="49">
+        <v>0</v>
+      </c>
+      <c r="C15" s="49">
+        <v>0</v>
+      </c>
+      <c r="D15" s="49">
+        <v>0</v>
+      </c>
+      <c r="E15" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="48" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" s="49">
+        <v>0</v>
+      </c>
+      <c r="C16" s="49">
+        <v>0</v>
+      </c>
+      <c r="D16" s="49">
+        <v>0</v>
+      </c>
+      <c r="E16" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="48" t="s">
+        <v>68</v>
+      </c>
+      <c r="B17" s="49">
+        <v>0</v>
+      </c>
+      <c r="C17" s="49">
+        <v>0</v>
+      </c>
+      <c r="D17" s="49">
+        <v>0</v>
+      </c>
+      <c r="E17" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="48" t="s">
+        <v>70</v>
+      </c>
+      <c r="B18" s="49">
+        <v>0</v>
+      </c>
+      <c r="C18" s="49">
+        <v>0</v>
+      </c>
+      <c r="D18" s="49">
+        <v>0</v>
+      </c>
+      <c r="E18" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="48" t="s">
+        <v>110</v>
+      </c>
+      <c r="B19" s="49">
+        <v>0</v>
+      </c>
+      <c r="C19" s="49">
+        <v>0</v>
+      </c>
+      <c r="D19" s="49">
+        <v>0</v>
+      </c>
+      <c r="E19" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="48" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="49">
+        <v>0</v>
+      </c>
+      <c r="C20" s="49">
+        <v>0</v>
+      </c>
+      <c r="D20" s="49">
+        <v>0</v>
+      </c>
+      <c r="E20" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="48" t="s">
+        <v>77</v>
+      </c>
+      <c r="B21" s="49">
+        <v>0</v>
+      </c>
+      <c r="C21" s="49">
+        <v>0</v>
+      </c>
+      <c r="D21" s="49">
+        <v>0</v>
+      </c>
+      <c r="E21" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="48" t="s">
+        <v>78</v>
+      </c>
+      <c r="B22" s="49">
+        <v>0</v>
+      </c>
+      <c r="C22" s="49">
+        <v>0</v>
+      </c>
+      <c r="D22" s="49">
+        <v>0</v>
+      </c>
+      <c r="E22" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="48" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="49">
+        <v>0</v>
+      </c>
+      <c r="C23" s="49">
+        <v>0</v>
+      </c>
+      <c r="D23" s="49">
+        <v>0</v>
+      </c>
+      <c r="E23" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" s="48" t="s">
+        <v>80</v>
+      </c>
+      <c r="B24" s="49">
+        <v>0</v>
+      </c>
+      <c r="C24" s="49">
+        <v>0</v>
+      </c>
+      <c r="D24" s="49">
+        <v>0</v>
+      </c>
+      <c r="E24" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" s="48" t="s">
+        <v>82</v>
+      </c>
+      <c r="B25" s="49">
+        <v>0</v>
+      </c>
+      <c r="C25" s="49">
+        <v>0</v>
+      </c>
+      <c r="D25" s="49">
+        <v>0</v>
+      </c>
+      <c r="E25" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" s="48" t="s">
+        <v>83</v>
+      </c>
+      <c r="B26" s="49">
+        <v>0</v>
+      </c>
+      <c r="C26" s="49">
+        <v>0</v>
+      </c>
+      <c r="D26" s="49">
+        <v>0.48958400000000002</v>
+      </c>
+      <c r="E26" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" s="48" t="s">
+        <v>88</v>
+      </c>
+      <c r="B27" s="49">
+        <v>0</v>
+      </c>
+      <c r="C27" s="49">
+        <v>0</v>
+      </c>
+      <c r="D27" s="49">
+        <v>0</v>
+      </c>
+      <c r="E27" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" s="48" t="s">
+        <v>89</v>
+      </c>
+      <c r="B28" s="49">
+        <v>0</v>
+      </c>
+      <c r="C28" s="49">
+        <v>0</v>
+      </c>
+      <c r="D28" s="49">
+        <v>0</v>
+      </c>
+      <c r="E28" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="48" t="s">
+        <v>96</v>
+      </c>
+      <c r="B29" s="49">
+        <v>0</v>
+      </c>
+      <c r="C29" s="49">
+        <v>0</v>
+      </c>
+      <c r="D29" s="49">
+        <v>0.160417</v>
+      </c>
+      <c r="E29" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" s="48" t="s">
         <v>99</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="B30" s="49">
+        <v>0</v>
+      </c>
+      <c r="C30" s="49">
+        <v>0</v>
+      </c>
+      <c r="D30" s="49">
+        <v>0</v>
+      </c>
+      <c r="E30" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" s="48" t="s">
         <v>100</v>
       </c>
-      <c r="D6" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="E6" s="6" t="s">
+      <c r="B31" s="49">
+        <v>0</v>
+      </c>
+      <c r="C31" s="49">
+        <v>0</v>
+      </c>
+      <c r="D31" s="49">
+        <v>0</v>
+      </c>
+      <c r="E31" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" s="48" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="7">
-        <v>0</v>
-      </c>
-      <c r="C7" s="7">
-        <v>0</v>
-      </c>
-      <c r="D7" s="7">
-        <v>0</v>
-      </c>
-      <c r="E7" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="7">
-        <v>0</v>
-      </c>
-      <c r="C8" s="7">
-        <v>0</v>
-      </c>
-      <c r="D8" s="7">
-        <v>0</v>
-      </c>
-      <c r="E8" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="7">
-        <v>0</v>
-      </c>
-      <c r="C9" s="7">
-        <v>0</v>
-      </c>
-      <c r="D9" s="7">
-        <v>0</v>
-      </c>
-      <c r="E9" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" s="7">
-        <v>0</v>
-      </c>
-      <c r="C10" s="7">
-        <v>0</v>
-      </c>
-      <c r="D10" s="7">
-        <v>0</v>
-      </c>
-      <c r="E10" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" s="7">
-        <v>0</v>
-      </c>
-      <c r="C11" s="7">
-        <v>0</v>
-      </c>
-      <c r="D11" s="7">
-        <v>0</v>
-      </c>
-      <c r="E11" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B12" s="7">
-        <v>0</v>
-      </c>
-      <c r="C12" s="7">
-        <v>0</v>
-      </c>
-      <c r="D12" s="7">
-        <v>0</v>
-      </c>
-      <c r="E12" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="7">
-        <v>0</v>
-      </c>
-      <c r="C13" s="7">
-        <v>0</v>
-      </c>
-      <c r="D13" s="7">
-        <v>0</v>
-      </c>
-      <c r="E13" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="B14" s="7">
-        <v>0</v>
-      </c>
-      <c r="C14" s="7">
-        <v>0</v>
-      </c>
-      <c r="D14" s="7">
-        <v>0</v>
-      </c>
-      <c r="E14" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B15" s="7">
-        <v>0</v>
-      </c>
-      <c r="C15" s="7">
-        <v>0</v>
-      </c>
-      <c r="D15" s="7">
-        <v>0</v>
-      </c>
-      <c r="E15" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="B16" s="7">
-        <v>0</v>
-      </c>
-      <c r="C16" s="7">
-        <v>0</v>
-      </c>
-      <c r="D16" s="7">
-        <v>0</v>
-      </c>
-      <c r="E16" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="B17" s="7">
-        <v>0</v>
-      </c>
-      <c r="C17" s="7">
-        <v>0</v>
-      </c>
-      <c r="D17" s="7">
-        <v>0</v>
-      </c>
-      <c r="E17" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="B18" s="7">
-        <v>0</v>
-      </c>
-      <c r="C18" s="7">
-        <v>0</v>
-      </c>
-      <c r="D18" s="7">
-        <v>0</v>
-      </c>
-      <c r="E18" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B19" s="7">
-        <v>0</v>
-      </c>
-      <c r="C19" s="7">
-        <v>0</v>
-      </c>
-      <c r="D19" s="7">
-        <v>0</v>
-      </c>
-      <c r="E19" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="B20" s="7">
-        <v>0</v>
-      </c>
-      <c r="C20" s="7">
-        <v>0</v>
-      </c>
-      <c r="D20" s="7">
-        <v>0</v>
-      </c>
-      <c r="E20" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="B21" s="7">
-        <v>0</v>
-      </c>
-      <c r="C21" s="7">
-        <v>0</v>
-      </c>
-      <c r="D21" s="7">
-        <v>0</v>
-      </c>
-      <c r="E21" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B22" s="7">
-        <v>0</v>
-      </c>
-      <c r="C22" s="7">
-        <v>0</v>
-      </c>
-      <c r="D22" s="7">
-        <v>0</v>
-      </c>
-      <c r="E22" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B23" s="7">
-        <v>0</v>
-      </c>
-      <c r="C23" s="7">
-        <v>0</v>
-      </c>
-      <c r="D23" s="7">
-        <v>0</v>
-      </c>
-      <c r="E23" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B24" s="7">
-        <v>0</v>
-      </c>
-      <c r="C24" s="7">
-        <v>0</v>
-      </c>
-      <c r="D24" s="7">
-        <v>0</v>
-      </c>
-      <c r="E24" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B25" s="7">
-        <v>0</v>
-      </c>
-      <c r="C25" s="7">
-        <v>0</v>
-      </c>
-      <c r="D25" s="7">
-        <v>0</v>
-      </c>
-      <c r="E25" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="B26" s="7">
-        <v>0</v>
-      </c>
-      <c r="C26" s="7">
-        <v>0</v>
-      </c>
-      <c r="D26" s="7">
-        <v>0.48958400000000002</v>
-      </c>
-      <c r="E26" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="B27" s="7">
-        <v>0</v>
-      </c>
-      <c r="C27" s="7">
-        <v>0</v>
-      </c>
-      <c r="D27" s="7">
-        <v>0</v>
-      </c>
-      <c r="E27" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B28" s="7">
-        <v>0</v>
-      </c>
-      <c r="C28" s="7">
-        <v>0</v>
-      </c>
-      <c r="D28" s="7">
-        <v>0</v>
-      </c>
-      <c r="E28" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="B29" s="7">
-        <v>0</v>
-      </c>
-      <c r="C29" s="7">
-        <v>0</v>
-      </c>
-      <c r="D29" s="7">
-        <v>0.160417</v>
-      </c>
-      <c r="E29" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B30" s="7">
-        <v>0</v>
-      </c>
-      <c r="C30" s="7">
-        <v>0</v>
-      </c>
-      <c r="D30" s="7">
-        <v>0</v>
-      </c>
-      <c r="E30" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="B31" s="7">
-        <v>0</v>
-      </c>
-      <c r="C31" s="7">
-        <v>0</v>
-      </c>
-      <c r="D31" s="7">
-        <v>0</v>
-      </c>
-      <c r="E31" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="B32" s="7">
-        <v>0</v>
-      </c>
-      <c r="C32" s="7">
-        <v>0</v>
-      </c>
-      <c r="D32" s="7">
-        <v>0</v>
-      </c>
-      <c r="E32" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B33" s="8">
-        <v>0</v>
-      </c>
-      <c r="C33" s="8">
-        <v>0</v>
-      </c>
-      <c r="D33" s="8">
+      <c r="B32" s="49">
+        <v>0</v>
+      </c>
+      <c r="C32" s="49">
+        <v>0</v>
+      </c>
+      <c r="D32" s="49">
+        <v>0</v>
+      </c>
+      <c r="E32" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5">
+      <c r="B33" s="50">
+        <v>0</v>
+      </c>
+      <c r="C33" s="50">
+        <v>0</v>
+      </c>
+      <c r="D33" s="50">
         <v>0.65</v>
       </c>
-      <c r="E33" s="8">
+      <c r="E33" s="50">
         <v>0</v>
       </c>
     </row>
@@ -6433,49 +6394,49 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+    <row r="1" spans="1:2" ht="15.75">
+      <c r="A1" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="B4" s="11" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="B5" s="11"/>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>110</v>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="B4" s="52" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="51" t="s">
+        <v>113</v>
+      </c>
+      <c r="B5" s="52"/>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="51" t="s">
+        <v>114</v>
+      </c>
+      <c r="B6" s="52" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="51" t="s">
+        <v>115</v>
+      </c>
+      <c r="B7" s="52" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="51" t="s">
+        <v>117</v>
+      </c>
+      <c r="B8" s="52" t="s">
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -6485,6 +6446,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3c298670-db79-47a5-968d-a4570c34317f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="17e8e7ea-beb0-4155-adc4-5bfa61f32508" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F57AE488C1C9C348AE667C65EC1B6349" ma:contentTypeVersion="84" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="7ffe0223de2040b214974ba9767dc658">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3c298670-db79-47a5-968d-a4570c34317f" xmlns:ns3="17e8e7ea-beb0-4155-adc4-5bfa61f32508" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0b0806029c900830a7d915fa99f226c3" ns2:_="" ns3:_="">
     <xsd:import namespace="3c298670-db79-47a5-968d-a4570c34317f"/>
@@ -6635,28 +6616,8 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3c298670-db79-47a5-968d-a4570c34317f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="17e8e7ea-beb0-4155-adc4-5bfa61f32508" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D598798-BEAE-4153-B302-5E39E634C73F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1CA6D523-C467-48E4-8347-A52F87752CEA}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6664,5 +6625,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1CA6D523-C467-48E4-8347-A52F87752CEA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D598798-BEAE-4153-B302-5E39E634C73F}"/>
 </file>
</xml_diff>